<commit_message>
feat: Nouveau module Mésure Mensuelle avec export Excel et gestion des conflits de fichiers Excel locaux
</commit_message>
<xml_diff>
--- a/MESURE_NAVIRES_2026.xlsx
+++ b/MESURE_NAVIRES_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\AntiGravity\gestion_des_navires\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F8830E-DCA9-4DEA-90DA-1B05E8BC1D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F879F252-D2BC-4D8C-8D4B-DDC3981E4052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{F4F545B4-7D84-46B3-A660-206858AF8EC5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{F4F545B4-7D84-46B3-A660-206858AF8EC5}"/>
   </bookViews>
   <sheets>
     <sheet name="MESURE" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'AVRIL 2026'!$A$2:$L$14</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'FEVRIER 2026'!$A$2:$L$14</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'MARS 2026'!$A$2:$L$14</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'MARS 2026'!$A$2:$L$13</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">MESURE!$A$1:$K$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="72">
   <si>
     <t xml:space="preserve">NAVIRE  </t>
   </si>
@@ -258,17 +258,17 @@
     <t>DELAI DE TRANSMISSION DU FICHIER LE 03 DE CHAQUE MOIS  (FEVRIER 2026)</t>
   </si>
   <si>
-    <t>DELAI DE TRANSMISSION DU FICHIER LE 03 DE CHAQUE MOIS  (MARS 2026)</t>
-  </si>
-  <si>
     <t>DELAI DE TRANSMISSION DU FICHIER LE 03 DE CHAQUE MOIS  (AVRIL 2026)</t>
+  </si>
+  <si>
+    <t>MESURE "MARS 2026"</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -370,6 +370,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -397,7 +404,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="36">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -866,11 +873,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -984,24 +1004,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1085,44 +1087,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1171,6 +1137,78 @@
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
@@ -1523,18 +1561,18 @@
       <c r="A1" s="18"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
-      <c r="D1" s="41" t="s">
+      <c r="D1" s="85" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="41" t="s">
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="85" t="s">
         <v>60</v>
       </c>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="43"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="86"/>
+      <c r="K1" s="87"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
@@ -1810,71 +1848,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="90" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
+      <c r="A2" s="90"/>
+      <c r="B2" s="90"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="90"/>
+      <c r="H2" s="90"/>
+      <c r="I2" s="90"/>
+      <c r="J2" s="90"/>
+      <c r="K2" s="90"/>
+      <c r="L2" s="90"/>
     </row>
     <row r="3" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="46"/>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
+      <c r="A3" s="90"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
     </row>
     <row r="4" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.6">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
-      <c r="C4" s="45" t="s">
+      <c r="C4" s="89" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="44" t="s">
+      <c r="D4" s="89"/>
+      <c r="E4" s="89"/>
+      <c r="F4" s="89"/>
+      <c r="G4" s="88" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="44"/>
-      <c r="I4" s="44"/>
-      <c r="J4" s="44"/>
+      <c r="H4" s="88"/>
+      <c r="I4" s="88"/>
+      <c r="J4" s="88"/>
       <c r="K4" s="3"/>
     </row>
     <row r="5" spans="1:12" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="46" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="6" t="s">
@@ -1889,92 +1927,92 @@
       <c r="F5" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="56" t="s">
+      <c r="G5" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="57" t="s">
+      <c r="H5" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="57" t="s">
+      <c r="I5" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="J5" s="58" t="s">
+      <c r="J5" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="61" t="s">
+      <c r="K5" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="L5" s="62" t="s">
+      <c r="L5" s="56" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="55" t="s">
+      <c r="C6" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="55" t="s">
+      <c r="D6" s="49" t="s">
         <v>64</v>
       </c>
-      <c r="E6" s="55" t="s">
+      <c r="E6" s="49" t="s">
         <v>65</v>
       </c>
-      <c r="F6" s="55" t="s">
+      <c r="F6" s="49" t="s">
         <v>63</v>
       </c>
-      <c r="G6" s="59"/>
-      <c r="H6" s="60" t="s">
+      <c r="G6" s="53"/>
+      <c r="H6" s="54" t="s">
         <v>66</v>
       </c>
-      <c r="I6" s="60" t="s">
+      <c r="I6" s="54" t="s">
         <v>67</v>
       </c>
-      <c r="J6" s="60" t="s">
+      <c r="J6" s="54" t="s">
         <v>68</v>
       </c>
-      <c r="K6" s="63"/>
-      <c r="L6" s="64"/>
+      <c r="K6" s="57"/>
+      <c r="L6" s="58"/>
     </row>
     <row r="7" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="47" t="s">
+      <c r="A7" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="49">
+      <c r="C7" s="43">
         <v>46059</v>
       </c>
-      <c r="D7" s="49">
+      <c r="D7" s="43">
         <v>46048</v>
       </c>
-      <c r="E7" s="49">
+      <c r="E7" s="43">
         <v>46048</v>
       </c>
-      <c r="F7" s="49">
+      <c r="F7" s="43">
         <v>46055</v>
       </c>
-      <c r="G7" s="49">
+      <c r="G7" s="43">
         <v>46054</v>
       </c>
-      <c r="H7" s="50" t="s">
+      <c r="H7" s="44" t="s">
         <v>36</v>
       </c>
-      <c r="I7" s="50" t="s">
+      <c r="I7" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="J7" s="50" t="s">
+      <c r="J7" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="K7" s="50">
+      <c r="K7" s="44">
         <v>100</v>
       </c>
-      <c r="L7" s="50"/>
+      <c r="L7" s="44"/>
     </row>
     <row r="8" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
@@ -2316,7 +2354,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93CF256F-F55B-4A37-832D-0EB78B287215}">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.28515625" customWidth="1"/>
@@ -2328,208 +2366,188 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
-        <v>70</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
+      <c r="A1" s="90" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
+      <c r="A2" s="90"/>
+      <c r="B2" s="90"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="90"/>
+      <c r="H2" s="90"/>
+      <c r="I2" s="90"/>
+      <c r="J2" s="90"/>
+      <c r="K2" s="90"/>
+      <c r="L2" s="90"/>
     </row>
     <row r="3" spans="1:12" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="46"/>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
+      <c r="A3" s="90"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
     </row>
     <row r="4" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="85" t="s">
+      <c r="A4" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="85" t="s">
+      <c r="B4" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="74" t="s">
+      <c r="C4" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="78" t="s">
+      <c r="D4" s="92"/>
+      <c r="E4" s="92"/>
+      <c r="F4" s="93"/>
+      <c r="G4" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="76"/>
-      <c r="I4" s="76"/>
-      <c r="J4" s="77"/>
-      <c r="K4" s="83" t="s">
+      <c r="H4" s="95"/>
+      <c r="I4" s="95"/>
+      <c r="J4" s="96"/>
+      <c r="K4" s="97" t="s">
         <v>18</v>
       </c>
-      <c r="L4" s="81" t="s">
+      <c r="L4" s="99" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="86"/>
-      <c r="B5" s="86"/>
-      <c r="C5" s="95" t="s">
+      <c r="A5" s="102"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="96" t="s">
+      <c r="D5" s="103" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="98" t="s">
+      <c r="E5" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="97" t="s">
+      <c r="F5" s="104" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="99" t="s">
+      <c r="G5" s="105" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="100" t="s">
+      <c r="H5" s="82" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="101" t="s">
+      <c r="I5" s="106" t="s">
         <v>11</v>
       </c>
-      <c r="J5" s="100" t="s">
+      <c r="J5" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="84"/>
-      <c r="L5" s="82"/>
-    </row>
-    <row r="6" spans="1:12" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="87" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="88" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="89" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="90" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" s="89" t="s">
-        <v>65</v>
-      </c>
-      <c r="F6" s="90" t="s">
-        <v>63</v>
-      </c>
-      <c r="G6" s="91" t="s">
-        <v>5</v>
-      </c>
-      <c r="H6" s="92" t="s">
-        <v>66</v>
-      </c>
-      <c r="I6" s="93" t="s">
-        <v>67</v>
-      </c>
-      <c r="J6" s="92" t="s">
-        <v>68</v>
-      </c>
-      <c r="K6" s="80"/>
-      <c r="L6" s="94"/>
+      <c r="K5" s="98"/>
+      <c r="L5" s="100"/>
+    </row>
+    <row r="6" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="84"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="43"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="60"/>
     </row>
     <row r="7" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="65"/>
-      <c r="B7" s="48"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
-      <c r="I7" s="50"/>
-      <c r="J7" s="50"/>
-      <c r="K7" s="50"/>
-      <c r="L7" s="66"/>
+      <c r="A7" s="39"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="38"/>
     </row>
     <row r="8" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="39"/>
+      <c r="A8" s="40"/>
       <c r="B8" s="9"/>
       <c r="C8" s="11"/>
       <c r="D8" s="12"/>
       <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
+      <c r="F8" s="11"/>
       <c r="G8" s="11"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
       <c r="K8" s="12"/>
       <c r="L8" s="38"/>
     </row>
     <row r="9" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="40"/>
+      <c r="A9" s="39"/>
       <c r="B9" s="9"/>
       <c r="C9" s="11"/>
       <c r="D9" s="12"/>
       <c r="E9" s="12"/>
-      <c r="F9" s="11"/>
+      <c r="F9" s="12"/>
       <c r="G9" s="11"/>
       <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
+      <c r="I9" s="12"/>
       <c r="J9" s="11"/>
       <c r="K9" s="12"/>
       <c r="L9" s="38"/>
     </row>
     <row r="10" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="39"/>
+      <c r="A10" s="40"/>
       <c r="B10" s="9"/>
       <c r="C10" s="11"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
       <c r="I10" s="12"/>
-      <c r="J10" s="11"/>
+      <c r="J10" s="12"/>
       <c r="K10" s="12"/>
       <c r="L10" s="38"/>
     </row>
     <row r="11" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="40"/>
+      <c r="A11" s="39"/>
       <c r="B11" s="9"/>
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
       <c r="F11" s="11"/>
-      <c r="G11" s="12"/>
+      <c r="G11" s="11"/>
       <c r="H11" s="12"/>
       <c r="I11" s="12"/>
       <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="38"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="61"/>
     </row>
     <row r="12" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="39"/>
@@ -2539,23 +2557,23 @@
       <c r="E12" s="11"/>
       <c r="F12" s="11"/>
       <c r="G12" s="11"/>
-      <c r="H12" s="12"/>
+      <c r="H12" s="11"/>
       <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="67"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="38"/>
     </row>
     <row r="13" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="39"/>
       <c r="B13" s="9"/>
       <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
+      <c r="D13" s="12"/>
       <c r="E13" s="11"/>
       <c r="F13" s="11"/>
       <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
+      <c r="H13" s="12"/>
       <c r="I13" s="12"/>
-      <c r="J13" s="11"/>
+      <c r="J13" s="12"/>
       <c r="K13" s="12"/>
       <c r="L13" s="38"/>
     </row>
@@ -2564,42 +2582,28 @@
       <c r="B14" s="9"/>
       <c r="C14" s="11"/>
       <c r="D14" s="12"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
       <c r="G14" s="11"/>
-      <c r="H14" s="12"/>
+      <c r="H14" s="11"/>
       <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
+      <c r="J14" s="11"/>
       <c r="K14" s="12"/>
       <c r="L14" s="38"/>
     </row>
-    <row r="15" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="39"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="12"/>
-      <c r="L15" s="38"/>
-    </row>
-    <row r="16" spans="1:12" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="68"/>
-      <c r="B16" s="69"/>
-      <c r="C16" s="70"/>
-      <c r="D16" s="70"/>
-      <c r="E16" s="70"/>
-      <c r="F16" s="70"/>
-      <c r="G16" s="71"/>
-      <c r="H16" s="72"/>
-      <c r="I16" s="72"/>
-      <c r="J16" s="72"/>
-      <c r="K16" s="72"/>
-      <c r="L16" s="73"/>
+    <row r="15" spans="1:12" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="62"/>
+      <c r="B15" s="63"/>
+      <c r="C15" s="64"/>
+      <c r="D15" s="64"/>
+      <c r="E15" s="64"/>
+      <c r="F15" s="64"/>
+      <c r="G15" s="65"/>
+      <c r="H15" s="66"/>
+      <c r="I15" s="66"/>
+      <c r="J15" s="66"/>
+      <c r="K15" s="66"/>
+      <c r="L15" s="67"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2633,152 +2637,152 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="46" t="s">
-        <v>71</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="I1" s="46"/>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
+      <c r="A1" s="90" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
     </row>
     <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46"/>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
+      <c r="A2" s="90"/>
+      <c r="B2" s="90"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="90"/>
+      <c r="E2" s="90"/>
+      <c r="F2" s="90"/>
+      <c r="G2" s="90"/>
+      <c r="H2" s="90"/>
+      <c r="I2" s="90"/>
+      <c r="J2" s="90"/>
+      <c r="K2" s="90"/>
+      <c r="L2" s="90"/>
     </row>
     <row r="3" spans="1:12" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="46"/>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
+      <c r="A3" s="90"/>
+      <c r="B3" s="90"/>
+      <c r="C3" s="90"/>
+      <c r="D3" s="90"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="90"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="90"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
     </row>
     <row r="4" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="85" t="s">
+      <c r="A4" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="85" t="s">
+      <c r="B4" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="74" t="s">
+      <c r="C4" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="78" t="s">
+      <c r="D4" s="92"/>
+      <c r="E4" s="92"/>
+      <c r="F4" s="93"/>
+      <c r="G4" s="94" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="76"/>
-      <c r="I4" s="76"/>
-      <c r="J4" s="77"/>
-      <c r="K4" s="83" t="s">
+      <c r="H4" s="95"/>
+      <c r="I4" s="95"/>
+      <c r="J4" s="96"/>
+      <c r="K4" s="97" t="s">
         <v>18</v>
       </c>
-      <c r="L4" s="81" t="s">
+      <c r="L4" s="99" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="86"/>
-      <c r="B5" s="86"/>
-      <c r="C5" s="95" t="s">
+      <c r="A5" s="102"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="96" t="s">
+      <c r="D5" s="78" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="98" t="s">
+      <c r="E5" s="80" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="97" t="s">
+      <c r="F5" s="79" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="99" t="s">
+      <c r="G5" s="81" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="100" t="s">
+      <c r="H5" s="82" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="101" t="s">
+      <c r="I5" s="83" t="s">
         <v>11</v>
       </c>
-      <c r="J5" s="100" t="s">
+      <c r="J5" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="84"/>
-      <c r="L5" s="82"/>
+      <c r="K5" s="98"/>
+      <c r="L5" s="100"/>
     </row>
     <row r="6" spans="1:12" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="87" t="s">
+      <c r="A6" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="88" t="s">
+      <c r="B6" s="70" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="89" t="s">
+      <c r="C6" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="90" t="s">
+      <c r="D6" s="72" t="s">
         <v>64</v>
       </c>
-      <c r="E6" s="89" t="s">
+      <c r="E6" s="71" t="s">
         <v>65</v>
       </c>
-      <c r="F6" s="90" t="s">
+      <c r="F6" s="72" t="s">
         <v>63</v>
       </c>
-      <c r="G6" s="91" t="s">
+      <c r="G6" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="92" t="s">
+      <c r="H6" s="74" t="s">
         <v>66</v>
       </c>
-      <c r="I6" s="93" t="s">
+      <c r="I6" s="75" t="s">
         <v>67</v>
       </c>
-      <c r="J6" s="92" t="s">
+      <c r="J6" s="74" t="s">
         <v>68</v>
       </c>
-      <c r="K6" s="80"/>
-      <c r="L6" s="94"/>
+      <c r="K6" s="68"/>
+      <c r="L6" s="76"/>
     </row>
     <row r="7" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="65"/>
-      <c r="B7" s="48"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="50"/>
-      <c r="I7" s="50"/>
-      <c r="J7" s="50"/>
-      <c r="K7" s="50"/>
-      <c r="L7" s="66"/>
+      <c r="A7" s="59"/>
+      <c r="B7" s="42"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="60"/>
     </row>
     <row r="8" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="39"/>
@@ -2848,7 +2852,7 @@
       <c r="I12" s="12"/>
       <c r="J12" s="12"/>
       <c r="K12" s="14"/>
-      <c r="L12" s="67"/>
+      <c r="L12" s="61"/>
     </row>
     <row r="13" spans="1:12" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="39"/>
@@ -2893,18 +2897,18 @@
       <c r="L15" s="38"/>
     </row>
     <row r="16" spans="1:12" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="68"/>
-      <c r="B16" s="69"/>
-      <c r="C16" s="70"/>
-      <c r="D16" s="70"/>
-      <c r="E16" s="70"/>
-      <c r="F16" s="70"/>
-      <c r="G16" s="71"/>
-      <c r="H16" s="72"/>
-      <c r="I16" s="72"/>
-      <c r="J16" s="72"/>
-      <c r="K16" s="72"/>
-      <c r="L16" s="73"/>
+      <c r="A16" s="62"/>
+      <c r="B16" s="63"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="64"/>
+      <c r="G16" s="65"/>
+      <c r="H16" s="66"/>
+      <c r="I16" s="66"/>
+      <c r="J16" s="66"/>
+      <c r="K16" s="66"/>
+      <c r="L16" s="67"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>